<commit_message>
Auto-conversión de datos meteorológicos a CSV y XLSX
</commit_message>
<xml_diff>
--- a/downld02.xlsx
+++ b/downld02.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL37"/>
+  <dimension ref="A1:AH37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -514,10 +514,6 @@
     <col width="13" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="13" customWidth="1" min="34" max="34"/>
-    <col width="13" customWidth="1" min="35" max="35"/>
-    <col width="13" customWidth="1" min="36" max="36"/>
-    <col width="13" customWidth="1" min="37" max="37"/>
-    <col width="13" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,119 +525,175 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="R3" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="S3" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="T3" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="U3" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="V3" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="W3" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="X3" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="Y3" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="Z3" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="AA3" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="AB3" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="AC3" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="AD3" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="AE3" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="AF3" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="AG3" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="AH3" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="AI3" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="AJ3" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="AK3" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="AL3" s="2" t="n">
-        <v>37</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Temp Ext (°C)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Temp Máx</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Temp Mín</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Humedad Ext (%)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Punto Rocío</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Vel Vent</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Dir Vent</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Ráfaga Vent</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Vel Máx</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Dir Máx</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Sens Term Wind</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Índice Calor</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>THW</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>THSW</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Presión (hPa)</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Lluvia (mm)</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Int Lluvia</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>Rad Solar</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Energía Solar</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Rad Solar Máx</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>UV</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>Dosis UV</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>UV Máx</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>Grados Día C</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>Grados Día F</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>Temp Int</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>Humedad Int</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>ET</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>Muestras Vent</t>
+        </is>
+      </c>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Tx Vent</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Recepción ISS</t>
+        </is>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Intervalo Arc</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -757,18 +809,6 @@
       <c r="AH4" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI4" s="5" t="n">
-        <v>1358</v>
-      </c>
-      <c r="AJ4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK4" s="4" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="AL4" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -883,18 +923,6 @@
       <c r="AH5" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI5" s="8" t="n">
-        <v>1356</v>
-      </c>
-      <c r="AJ5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK5" s="7" t="n">
-        <v>99.09999999999999</v>
-      </c>
-      <c r="AL5" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1009,18 +1037,6 @@
       <c r="AH6" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI6" s="5" t="n">
-        <v>1364</v>
-      </c>
-      <c r="AJ6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK6" s="4" t="n">
-        <v>99.7</v>
-      </c>
-      <c r="AL6" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -1135,18 +1151,6 @@
       <c r="AH7" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI7" s="8" t="n">
-        <v>1361</v>
-      </c>
-      <c r="AJ7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK7" s="7" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="AL7" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1261,18 +1265,6 @@
       <c r="AH8" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI8" s="5" t="n">
-        <v>1369</v>
-      </c>
-      <c r="AJ8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK8" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL8" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1387,18 +1379,6 @@
       <c r="AH9" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI9" s="8" t="n">
-        <v>1375</v>
-      </c>
-      <c r="AJ9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK9" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL9" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1513,18 +1493,6 @@
       <c r="AH10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AI10" s="5" t="n">
-        <v>1361</v>
-      </c>
-      <c r="AJ10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK10" s="4" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="AL10" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1639,18 +1607,6 @@
       <c r="AH11" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI11" s="8" t="n">
-        <v>1371</v>
-      </c>
-      <c r="AJ11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK11" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL11" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1765,18 +1721,6 @@
       <c r="AH12" s="4" t="n">
         <v>0.1</v>
       </c>
-      <c r="AI12" s="5" t="n">
-        <v>1369</v>
-      </c>
-      <c r="AJ12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK12" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL12" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1891,18 +1835,6 @@
       <c r="AH13" s="7" t="n">
         <v>0.28</v>
       </c>
-      <c r="AI13" s="8" t="n">
-        <v>1356</v>
-      </c>
-      <c r="AJ13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK13" s="7" t="n">
-        <v>99.09999999999999</v>
-      </c>
-      <c r="AL13" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2017,18 +1949,6 @@
       <c r="AH14" s="4" t="n">
         <v>0.33</v>
       </c>
-      <c r="AI14" s="5" t="n">
-        <v>1371</v>
-      </c>
-      <c r="AJ14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK14" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL14" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2143,18 +2063,6 @@
       <c r="AH15" s="7" t="n">
         <v>0.51</v>
       </c>
-      <c r="AI15" s="8" t="n">
-        <v>1372</v>
-      </c>
-      <c r="AJ15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK15" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL15" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2269,18 +2177,6 @@
       <c r="AH16" s="4" t="n">
         <v>0.61</v>
       </c>
-      <c r="AI16" s="5" t="n">
-        <v>1373</v>
-      </c>
-      <c r="AJ16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK16" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL16" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2395,18 +2291,6 @@
       <c r="AH17" s="7" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="AI17" s="8" t="n">
-        <v>1381</v>
-      </c>
-      <c r="AJ17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK17" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL17" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2521,18 +2405,6 @@
       <c r="AH18" s="4" t="n">
         <v>0.66</v>
       </c>
-      <c r="AI18" s="5" t="n">
-        <v>1389</v>
-      </c>
-      <c r="AJ18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK18" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL18" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -2647,18 +2519,6 @@
       <c r="AH19" s="7" t="n">
         <v>0.51</v>
       </c>
-      <c r="AI19" s="8" t="n">
-        <v>1379</v>
-      </c>
-      <c r="AJ19" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK19" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL19" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2773,18 +2633,6 @@
       <c r="AH20" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="AI20" s="5" t="n">
-        <v>1381</v>
-      </c>
-      <c r="AJ20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK20" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL20" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -2899,18 +2747,6 @@
       <c r="AH21" s="7" t="n">
         <v>0.15</v>
       </c>
-      <c r="AI21" s="8" t="n">
-        <v>1382</v>
-      </c>
-      <c r="AJ21" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK21" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL21" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -3025,18 +2861,6 @@
       <c r="AH22" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI22" s="5" t="n">
-        <v>1365</v>
-      </c>
-      <c r="AJ22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK22" s="4" t="n">
-        <v>99.8</v>
-      </c>
-      <c r="AL22" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -3151,18 +2975,6 @@
       <c r="AH23" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI23" s="8" t="n">
-        <v>1353</v>
-      </c>
-      <c r="AJ23" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK23" s="7" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="AL23" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -3277,18 +3089,6 @@
       <c r="AH24" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI24" s="5" t="n">
-        <v>1369</v>
-      </c>
-      <c r="AJ24" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK24" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL24" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -3403,18 +3203,6 @@
       <c r="AH25" s="7" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI25" s="8" t="n">
-        <v>1368</v>
-      </c>
-      <c r="AJ25" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK25" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL25" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3529,18 +3317,6 @@
       <c r="AH26" s="4" t="n">
         <v>0.08</v>
       </c>
-      <c r="AI26" s="5" t="n">
-        <v>1366</v>
-      </c>
-      <c r="AJ26" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK26" s="4" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="AL26" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -3655,18 +3431,6 @@
       <c r="AH27" s="7" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI27" s="8" t="n">
-        <v>1364</v>
-      </c>
-      <c r="AJ27" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK27" s="7" t="n">
-        <v>99.7</v>
-      </c>
-      <c r="AL27" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3781,18 +3545,6 @@
       <c r="AH28" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI28" s="5" t="n">
-        <v>1380</v>
-      </c>
-      <c r="AJ28" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK28" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL28" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -3907,18 +3659,6 @@
       <c r="AH29" s="7" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI29" s="8" t="n">
-        <v>1363</v>
-      </c>
-      <c r="AJ29" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK29" s="7" t="n">
-        <v>99.59999999999999</v>
-      </c>
-      <c r="AL29" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4033,18 +3773,6 @@
       <c r="AH30" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI30" s="5" t="n">
-        <v>1362</v>
-      </c>
-      <c r="AJ30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK30" s="4" t="n">
-        <v>99.59999999999999</v>
-      </c>
-      <c r="AL30" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -4159,18 +3887,6 @@
       <c r="AH31" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI31" s="8" t="n">
-        <v>1333</v>
-      </c>
-      <c r="AJ31" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK31" s="7" t="n">
-        <v>97.40000000000001</v>
-      </c>
-      <c r="AL31" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -4285,18 +4001,6 @@
       <c r="AH32" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI32" s="5" t="n">
-        <v>1323</v>
-      </c>
-      <c r="AJ32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK32" s="4" t="n">
-        <v>96.7</v>
-      </c>
-      <c r="AL32" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -4411,18 +4115,6 @@
       <c r="AH33" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI33" s="8" t="n">
-        <v>1358</v>
-      </c>
-      <c r="AJ33" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK33" s="7" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="AL33" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4537,18 +4229,6 @@
       <c r="AH34" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI34" s="5" t="n">
-        <v>1376</v>
-      </c>
-      <c r="AJ34" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK34" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="AL34" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -4663,18 +4343,6 @@
       <c r="AH35" s="7" t="n">
         <v>0.03</v>
       </c>
-      <c r="AI35" s="8" t="n">
-        <v>1353</v>
-      </c>
-      <c r="AJ35" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK35" s="7" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="AL35" s="8" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -4789,18 +4457,6 @@
       <c r="AH36" s="4" t="n">
         <v>0.13</v>
       </c>
-      <c r="AI36" s="5" t="n">
-        <v>1353</v>
-      </c>
-      <c r="AJ36" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK36" s="4" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="AL36" s="5" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -4914,18 +4570,6 @@
       </c>
       <c r="AH37" s="7" t="n">
         <v>0.2</v>
-      </c>
-      <c r="AI37" s="8" t="n">
-        <v>1361</v>
-      </c>
-      <c r="AJ37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK37" s="7" t="n">
-        <v>99.5</v>
-      </c>
-      <c r="AL37" s="8" t="n">
-        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>